<commit_message>
App 139 + change design table attr_value
</commit_message>
<xml_diff>
--- a/docs/test data.xlsx
+++ b/docs/test data.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JCCC\ArGlobal-1\Create-item-App\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52B76A0D-AF20-4BA5-889D-22EF4284895A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBF9E346-35DE-4F70-81EB-0A5F8F0C9E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{A100353F-A66F-4C9C-B0C4-57E4FE32D700}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="142">
   <si>
     <t>Item Type</t>
   </si>
@@ -289,13 +290,187 @@
   </si>
   <si>
     <t>None</t>
+  </si>
+  <si>
+    <t>General</t>
+  </si>
+  <si>
+    <t>Is it sent via PL/sql constant as of now. It will be a Profile Option</t>
+  </si>
+  <si>
+    <t>Profile Option</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is it sent via PL/sql constant as of now. It will be a Lookup </t>
+  </si>
+  <si>
+    <t>Lookup</t>
+  </si>
+  <si>
+    <t>Categories</t>
+  </si>
+  <si>
+    <t>Attributes - GRI</t>
+  </si>
+  <si>
+    <t>Attributes - MAS</t>
+  </si>
+  <si>
+    <t>Column heading</t>
+  </si>
+  <si>
+    <t>Where to see in EBS (App or Table)</t>
+  </si>
+  <si>
+    <t>ENGINEER (MAS)</t>
+  </si>
+  <si>
+    <t>F-5412-995</t>
+  </si>
+  <si>
+    <t>SUPER TEST 46 ADHESIVES F-5412-995</t>
+  </si>
+  <si>
+    <t>26-45</t>
+  </si>
+  <si>
+    <t>26-46</t>
+  </si>
+  <si>
+    <t>31.6 % SOLIDS; 7.5 LBS/GAL</t>
+  </si>
+  <si>
+    <t>Joel Calzadilla</t>
+  </si>
+  <si>
+    <t>ACRYLIC ADHESIVE</t>
+  </si>
+  <si>
+    <t>MAS, GRI</t>
+  </si>
+  <si>
+    <t>EL-94916-993</t>
+  </si>
+  <si>
+    <t>TFT</t>
+  </si>
+  <si>
+    <t>SUPER TEST 46 ADHESIVE_COATING EL-94916-993</t>
+  </si>
+  <si>
+    <t>PRECISION COATING</t>
+  </si>
+  <si>
+    <t>CV-8345-992</t>
+  </si>
+  <si>
+    <t>SUPER TEST 46 CONVERTING CV-8345-992</t>
+  </si>
+  <si>
+    <t>CUSTOM CONSTRUCTION</t>
+  </si>
+  <si>
+    <t>W-12005-992</t>
+  </si>
+  <si>
+    <t>SUPER TEST 46 LINER_COATING W-12005-992</t>
+  </si>
+  <si>
+    <t>LINER</t>
+  </si>
+  <si>
+    <t>R-13141-99</t>
+  </si>
+  <si>
+    <t>SUPER TEST 46 RAW_MATERIAL_ITEM R-13141-99</t>
+  </si>
+  <si>
+    <t>BACKING</t>
+  </si>
+  <si>
+    <t>FOOT</t>
+  </si>
+  <si>
+    <t>Slitting for CS</t>
+  </si>
+  <si>
+    <t>SP-9082-11</t>
+  </si>
+  <si>
+    <t>SUPER TEST 46 SLIT_CUSTOMER_SERVICE SP-9082-11</t>
+  </si>
+  <si>
+    <t>Splicing</t>
+  </si>
+  <si>
+    <t>SUPER TEST 46</t>
+  </si>
+  <si>
+    <t>NON-REPULPABLE ADHESIVE</t>
+  </si>
+  <si>
+    <t>Slitting for Eng</t>
+  </si>
+  <si>
+    <t>EL-94918-993</t>
+  </si>
+  <si>
+    <t>SUPER TEST 46 SLIT_ENGINEERING EL-94918-993</t>
+  </si>
+  <si>
+    <t>RUBBER ADHESIVE</t>
+  </si>
+  <si>
+    <t>F-5412-997</t>
+  </si>
+  <si>
+    <t>SUPER TEST 48 ADHESIVES F-5412-997</t>
+  </si>
+  <si>
+    <t>CV-8345-993</t>
+  </si>
+  <si>
+    <t>SUPER TEST 48 CONVERTING CV-8345-993</t>
+  </si>
+  <si>
+    <t>EL-94916-994</t>
+  </si>
+  <si>
+    <t>SUPER TEST 48 ADHESIVE_COATING EL-94916-994</t>
+  </si>
+  <si>
+    <t>W-12005-993</t>
+  </si>
+  <si>
+    <t>SUPER TEST 48 LINER_COATING W-12005-993</t>
+  </si>
+  <si>
+    <t>R-13142-01</t>
+  </si>
+  <si>
+    <t>SUPER TEST 48 RAW_MATERIAL_ITEM R-13142-01</t>
+  </si>
+  <si>
+    <t>SP-9082-12</t>
+  </si>
+  <si>
+    <t>SUPER TEST 48 SLIT_CUSTOMER_SERVICE SP-9082-12</t>
+  </si>
+  <si>
+    <t>SUPER TEST 48</t>
+  </si>
+  <si>
+    <t>EL-94918-994</t>
+  </si>
+  <si>
+    <t>SUPER TEST 48 SLIT_ENGINEERING EL-94918-994</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -318,6 +493,10 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Carlito"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -339,10 +518,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -677,7 +859,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAF3B785-2A61-40FA-87E9-F13F127C7845}">
-  <dimension ref="A1:AO6"/>
+  <dimension ref="A1:AX20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="16.1640625" bestFit="1" customWidth="1"/>
@@ -712,7 +894,7 @@
     <col min="40" max="40" width="19.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:41" s="2" customFormat="1">
+    <row r="1" spans="1:50" s="2" customFormat="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -837,7 +1019,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:41">
+    <row r="2" spans="1:50">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -893,7 +1075,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:41">
+    <row r="3" spans="1:50">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -937,7 +1119,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:41">
+    <row r="4" spans="1:50">
       <c r="A4" t="s">
         <v>40</v>
       </c>
@@ -1002,7 +1184,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:41">
+    <row r="5" spans="1:50">
       <c r="A5" t="s">
         <v>57</v>
       </c>
@@ -1040,7 +1222,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:41">
+    <row r="6" spans="1:50">
       <c r="A6" t="s">
         <v>63</v>
       </c>
@@ -1115,6 +1297,1556 @@
       </c>
       <c r="AO6" t="s">
         <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:50">
+      <c r="A7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I7" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="J7" s="3">
+        <v>230</v>
+      </c>
+      <c r="K7" s="3">
+        <v>31.6</v>
+      </c>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+      <c r="P7" s="3"/>
+      <c r="Q7" s="3"/>
+      <c r="R7" s="3"/>
+      <c r="S7" s="3"/>
+      <c r="T7" s="3"/>
+      <c r="U7" s="3"/>
+      <c r="V7" s="3">
+        <v>360</v>
+      </c>
+      <c r="W7" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="X7" s="3"/>
+      <c r="Y7" s="3">
+        <v>20</v>
+      </c>
+      <c r="Z7" s="3"/>
+      <c r="AA7" s="3">
+        <v>350</v>
+      </c>
+      <c r="AB7" s="3"/>
+      <c r="AC7" s="3"/>
+      <c r="AD7" s="3"/>
+      <c r="AE7" s="3"/>
+      <c r="AF7" s="3"/>
+      <c r="AG7" s="3"/>
+      <c r="AH7" s="3"/>
+      <c r="AI7" s="3"/>
+      <c r="AJ7" s="3"/>
+      <c r="AK7" s="3"/>
+      <c r="AL7" s="3"/>
+      <c r="AM7" s="3"/>
+      <c r="AN7" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AO7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="AP7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="AQ7" s="3"/>
+      <c r="AR7" s="3"/>
+      <c r="AS7" s="3"/>
+      <c r="AT7" s="3"/>
+      <c r="AU7" s="3"/>
+      <c r="AV7" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW7" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="AX7" s="3"/>
+    </row>
+    <row r="8" spans="1:50">
+      <c r="A8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N8" s="3">
+        <v>13</v>
+      </c>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3"/>
+      <c r="R8" s="3">
+        <v>180</v>
+      </c>
+      <c r="S8" s="3"/>
+      <c r="T8" s="3"/>
+      <c r="U8" s="3"/>
+      <c r="V8" s="3">
+        <v>360</v>
+      </c>
+      <c r="W8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="X8" s="3"/>
+      <c r="Y8" s="3">
+        <v>20</v>
+      </c>
+      <c r="Z8" s="3"/>
+      <c r="AA8" s="3"/>
+      <c r="AB8" s="3"/>
+      <c r="AC8" s="3"/>
+      <c r="AD8" s="3"/>
+      <c r="AE8" s="3"/>
+      <c r="AF8" s="3"/>
+      <c r="AG8" s="3"/>
+      <c r="AH8" s="3"/>
+      <c r="AI8" s="3"/>
+      <c r="AJ8" s="3"/>
+      <c r="AK8" s="3"/>
+      <c r="AL8" s="3"/>
+      <c r="AM8" s="3"/>
+      <c r="AN8" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AO8" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AP8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="AQ8" s="3"/>
+      <c r="AR8" s="3"/>
+      <c r="AS8" s="3"/>
+      <c r="AT8" s="3"/>
+      <c r="AU8" s="3"/>
+      <c r="AV8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW8" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="AX8" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9" spans="1:50">
+      <c r="A9" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
+      <c r="P9" s="3"/>
+      <c r="Q9" s="3"/>
+      <c r="R9" s="3"/>
+      <c r="S9" s="3"/>
+      <c r="T9" s="3"/>
+      <c r="U9" s="3"/>
+      <c r="V9" s="3">
+        <v>360</v>
+      </c>
+      <c r="W9" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="X9" s="3"/>
+      <c r="Y9" s="3">
+        <v>20</v>
+      </c>
+      <c r="Z9" s="3"/>
+      <c r="AA9" s="3"/>
+      <c r="AB9" s="3"/>
+      <c r="AC9" s="3"/>
+      <c r="AD9" s="3"/>
+      <c r="AE9" s="3"/>
+      <c r="AF9" s="3"/>
+      <c r="AG9" s="3"/>
+      <c r="AH9" s="3"/>
+      <c r="AI9" s="3"/>
+      <c r="AJ9" s="3"/>
+      <c r="AK9" s="3"/>
+      <c r="AL9" s="3"/>
+      <c r="AM9" s="3"/>
+      <c r="AN9" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AO9" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AP9" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="AQ9" s="3"/>
+      <c r="AR9" s="3"/>
+      <c r="AS9" s="3"/>
+      <c r="AT9" s="3"/>
+      <c r="AU9" s="3"/>
+      <c r="AV9" s="3"/>
+      <c r="AW9" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="AX9" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="10" spans="1:50">
+      <c r="A10" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N10" s="3"/>
+      <c r="O10" s="3"/>
+      <c r="P10" s="3"/>
+      <c r="Q10" s="3"/>
+      <c r="R10" s="3"/>
+      <c r="S10" s="3"/>
+      <c r="T10" s="3"/>
+      <c r="U10" s="3"/>
+      <c r="V10" s="3"/>
+      <c r="W10" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="X10" s="3"/>
+      <c r="Y10" s="3"/>
+      <c r="Z10" s="3"/>
+      <c r="AA10" s="3"/>
+      <c r="AB10" s="3"/>
+      <c r="AC10" s="3"/>
+      <c r="AD10" s="3"/>
+      <c r="AE10" s="3"/>
+      <c r="AF10" s="3"/>
+      <c r="AG10" s="3"/>
+      <c r="AH10" s="3"/>
+      <c r="AI10" s="3"/>
+      <c r="AJ10" s="3"/>
+      <c r="AK10" s="3"/>
+      <c r="AL10" s="3"/>
+      <c r="AM10" s="3"/>
+      <c r="AN10" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AO10" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AP10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="AQ10" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="AR10" s="3"/>
+      <c r="AS10" s="3"/>
+      <c r="AT10" s="3"/>
+      <c r="AU10" s="3"/>
+      <c r="AV10" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW10" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="AX10" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="11" spans="1:50">
+      <c r="A11" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="I11" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="J11" s="3">
+        <v>230</v>
+      </c>
+      <c r="K11" s="3">
+        <v>31.6</v>
+      </c>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N11" s="3"/>
+      <c r="O11" s="3"/>
+      <c r="P11" s="3"/>
+      <c r="Q11" s="3"/>
+      <c r="R11" s="3"/>
+      <c r="S11" s="3"/>
+      <c r="T11" s="3"/>
+      <c r="U11" s="3"/>
+      <c r="V11" s="3">
+        <v>360</v>
+      </c>
+      <c r="W11" s="3"/>
+      <c r="X11" s="3"/>
+      <c r="Y11" s="3">
+        <v>20</v>
+      </c>
+      <c r="Z11" s="3"/>
+      <c r="AA11" s="3"/>
+      <c r="AB11" s="3"/>
+      <c r="AC11" s="3"/>
+      <c r="AD11" s="3"/>
+      <c r="AE11" s="3"/>
+      <c r="AF11" s="3"/>
+      <c r="AG11" s="3">
+        <v>221</v>
+      </c>
+      <c r="AH11" s="3"/>
+      <c r="AI11" s="3"/>
+      <c r="AJ11" s="3"/>
+      <c r="AK11" s="3"/>
+      <c r="AL11" s="3"/>
+      <c r="AM11" s="3"/>
+      <c r="AN11" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AO11" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AP11" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="AQ11" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="AR11" s="3"/>
+      <c r="AS11" s="3"/>
+      <c r="AT11" s="3"/>
+      <c r="AU11" s="3"/>
+      <c r="AV11" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW11" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="AX11" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:50">
+      <c r="A12" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N12" s="3">
+        <v>13</v>
+      </c>
+      <c r="O12" s="3"/>
+      <c r="P12" s="3"/>
+      <c r="Q12" s="3"/>
+      <c r="R12" s="3">
+        <v>180</v>
+      </c>
+      <c r="S12" s="3"/>
+      <c r="T12" s="3"/>
+      <c r="U12" s="3"/>
+      <c r="V12" s="3">
+        <v>360</v>
+      </c>
+      <c r="W12" s="3"/>
+      <c r="X12" s="3"/>
+      <c r="Y12" s="3">
+        <v>20</v>
+      </c>
+      <c r="Z12" s="3"/>
+      <c r="AA12" s="3"/>
+      <c r="AB12" s="3"/>
+      <c r="AC12" s="3"/>
+      <c r="AD12" s="3"/>
+      <c r="AE12" s="3"/>
+      <c r="AF12" s="3"/>
+      <c r="AG12" s="3"/>
+      <c r="AH12" s="3"/>
+      <c r="AI12" s="3"/>
+      <c r="AJ12" s="3"/>
+      <c r="AK12" s="3"/>
+      <c r="AL12" s="3"/>
+      <c r="AM12" s="3"/>
+      <c r="AN12" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AO12" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AP12" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="AQ12" s="3"/>
+      <c r="AR12" s="3"/>
+      <c r="AS12" s="3"/>
+      <c r="AT12" s="3"/>
+      <c r="AU12" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="AV12" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW12" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="AX12" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="13" spans="1:50">
+      <c r="A13" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N13" s="3">
+        <v>13</v>
+      </c>
+      <c r="O13" s="3"/>
+      <c r="P13" s="3"/>
+      <c r="Q13" s="3"/>
+      <c r="R13" s="3">
+        <v>180</v>
+      </c>
+      <c r="S13" s="3"/>
+      <c r="T13" s="3"/>
+      <c r="U13" s="3"/>
+      <c r="V13" s="3">
+        <v>360</v>
+      </c>
+      <c r="W13" s="3"/>
+      <c r="X13" s="3"/>
+      <c r="Y13" s="3">
+        <v>20</v>
+      </c>
+      <c r="Z13" s="3"/>
+      <c r="AA13" s="3"/>
+      <c r="AB13" s="3"/>
+      <c r="AC13" s="3"/>
+      <c r="AD13" s="3"/>
+      <c r="AE13" s="3"/>
+      <c r="AF13" s="3"/>
+      <c r="AG13" s="3"/>
+      <c r="AH13" s="3"/>
+      <c r="AI13" s="3"/>
+      <c r="AJ13" s="3"/>
+      <c r="AK13" s="3"/>
+      <c r="AL13" s="3"/>
+      <c r="AM13" s="3"/>
+      <c r="AN13" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AO13" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AP13" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="AQ13" s="3"/>
+      <c r="AR13" s="3"/>
+      <c r="AS13" s="3"/>
+      <c r="AT13" s="3"/>
+      <c r="AU13" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="AV13" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW13" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="AX13" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="14" spans="1:50">
+      <c r="A14" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I14" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="J14" s="3">
+        <v>230</v>
+      </c>
+      <c r="K14" s="3">
+        <v>31.6</v>
+      </c>
+      <c r="L14" s="3"/>
+      <c r="M14" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N14" s="3"/>
+      <c r="O14" s="3"/>
+      <c r="P14" s="3"/>
+      <c r="Q14" s="3"/>
+      <c r="R14" s="3"/>
+      <c r="S14" s="3"/>
+      <c r="T14" s="3"/>
+      <c r="U14" s="3"/>
+      <c r="V14" s="3">
+        <v>360</v>
+      </c>
+      <c r="W14" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="X14" s="3"/>
+      <c r="Y14" s="3">
+        <v>20</v>
+      </c>
+      <c r="Z14" s="3"/>
+      <c r="AA14" s="3">
+        <v>350</v>
+      </c>
+      <c r="AB14" s="3"/>
+      <c r="AC14" s="3"/>
+      <c r="AD14" s="3"/>
+      <c r="AE14" s="3"/>
+      <c r="AF14" s="3"/>
+      <c r="AG14" s="3"/>
+      <c r="AH14" s="3"/>
+      <c r="AI14" s="3"/>
+      <c r="AJ14" s="3"/>
+      <c r="AK14" s="3"/>
+      <c r="AL14" s="3"/>
+      <c r="AM14" s="3"/>
+      <c r="AN14" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AO14" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AP14" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="AQ14" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="AR14" s="3"/>
+      <c r="AS14" s="3"/>
+      <c r="AT14" s="3"/>
+      <c r="AU14" s="3"/>
+      <c r="AV14" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW14" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="AX14" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="15" spans="1:50">
+      <c r="A15" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
+      <c r="M15" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N15" s="3">
+        <v>13</v>
+      </c>
+      <c r="O15" s="3"/>
+      <c r="P15" s="3"/>
+      <c r="Q15" s="3"/>
+      <c r="R15" s="3">
+        <v>180</v>
+      </c>
+      <c r="S15" s="3"/>
+      <c r="T15" s="3"/>
+      <c r="U15" s="3"/>
+      <c r="V15" s="3">
+        <v>360</v>
+      </c>
+      <c r="W15" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="X15" s="3"/>
+      <c r="Y15" s="3">
+        <v>20</v>
+      </c>
+      <c r="Z15" s="3"/>
+      <c r="AA15" s="3"/>
+      <c r="AB15" s="3"/>
+      <c r="AC15" s="3"/>
+      <c r="AD15" s="3"/>
+      <c r="AE15" s="3"/>
+      <c r="AF15" s="3"/>
+      <c r="AG15" s="3"/>
+      <c r="AH15" s="3"/>
+      <c r="AI15" s="3"/>
+      <c r="AJ15" s="3"/>
+      <c r="AK15" s="3"/>
+      <c r="AL15" s="3"/>
+      <c r="AM15" s="3"/>
+      <c r="AN15" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AO15" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AP15" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="AQ15" s="3"/>
+      <c r="AR15" s="3"/>
+      <c r="AS15" s="3"/>
+      <c r="AT15" s="3"/>
+      <c r="AU15" s="3"/>
+      <c r="AV15" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW15" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="AX15" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="16" spans="1:50">
+      <c r="A16" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
+      <c r="M16" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N16" s="3"/>
+      <c r="O16" s="3"/>
+      <c r="P16" s="3"/>
+      <c r="Q16" s="3"/>
+      <c r="R16" s="3"/>
+      <c r="S16" s="3"/>
+      <c r="T16" s="3"/>
+      <c r="U16" s="3"/>
+      <c r="V16" s="3">
+        <v>360</v>
+      </c>
+      <c r="W16" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="X16" s="3"/>
+      <c r="Y16" s="3">
+        <v>20</v>
+      </c>
+      <c r="Z16" s="3"/>
+      <c r="AA16" s="3"/>
+      <c r="AB16" s="3"/>
+      <c r="AC16" s="3"/>
+      <c r="AD16" s="3"/>
+      <c r="AE16" s="3"/>
+      <c r="AF16" s="3"/>
+      <c r="AG16" s="3"/>
+      <c r="AH16" s="3"/>
+      <c r="AI16" s="3"/>
+      <c r="AJ16" s="3"/>
+      <c r="AK16" s="3"/>
+      <c r="AL16" s="3"/>
+      <c r="AM16" s="3"/>
+      <c r="AN16" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AO16" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AP16" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="AQ16" s="3"/>
+      <c r="AR16" s="3"/>
+      <c r="AS16" s="3"/>
+      <c r="AT16" s="3"/>
+      <c r="AU16" s="3"/>
+      <c r="AV16" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW16" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="AX16" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="17" spans="1:50">
+      <c r="A17" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+      <c r="M17" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N17" s="3"/>
+      <c r="O17" s="3"/>
+      <c r="P17" s="3"/>
+      <c r="Q17" s="3"/>
+      <c r="R17" s="3"/>
+      <c r="S17" s="3"/>
+      <c r="T17" s="3"/>
+      <c r="U17" s="3"/>
+      <c r="V17" s="3">
+        <v>360</v>
+      </c>
+      <c r="W17" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="X17" s="3"/>
+      <c r="Y17" s="3"/>
+      <c r="Z17" s="3"/>
+      <c r="AA17" s="3"/>
+      <c r="AB17" s="3"/>
+      <c r="AC17" s="3"/>
+      <c r="AD17" s="3"/>
+      <c r="AE17" s="3"/>
+      <c r="AF17" s="3"/>
+      <c r="AG17" s="3"/>
+      <c r="AH17" s="3"/>
+      <c r="AI17" s="3"/>
+      <c r="AJ17" s="3"/>
+      <c r="AK17" s="3"/>
+      <c r="AL17" s="3"/>
+      <c r="AM17" s="3"/>
+      <c r="AN17" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AO17" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AP17" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="AQ17" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="AR17" s="3"/>
+      <c r="AS17" s="3"/>
+      <c r="AT17" s="3"/>
+      <c r="AU17" s="3"/>
+      <c r="AV17" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW17" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="AX17" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="18" spans="1:50">
+      <c r="A18" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="I18" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="J18" s="3">
+        <v>230</v>
+      </c>
+      <c r="K18" s="3">
+        <v>31.6</v>
+      </c>
+      <c r="L18" s="3"/>
+      <c r="M18" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N18" s="3"/>
+      <c r="O18" s="3"/>
+      <c r="P18" s="3"/>
+      <c r="Q18" s="3"/>
+      <c r="R18" s="3"/>
+      <c r="S18" s="3"/>
+      <c r="T18" s="3"/>
+      <c r="U18" s="3"/>
+      <c r="V18" s="3">
+        <v>360</v>
+      </c>
+      <c r="W18" s="3"/>
+      <c r="X18" s="3"/>
+      <c r="Y18" s="3">
+        <v>20</v>
+      </c>
+      <c r="Z18" s="3"/>
+      <c r="AA18" s="3"/>
+      <c r="AB18" s="3"/>
+      <c r="AC18" s="3"/>
+      <c r="AD18" s="3"/>
+      <c r="AE18" s="3"/>
+      <c r="AF18" s="3"/>
+      <c r="AG18" s="3">
+        <v>221</v>
+      </c>
+      <c r="AH18" s="3"/>
+      <c r="AI18" s="3"/>
+      <c r="AJ18" s="3"/>
+      <c r="AK18" s="3"/>
+      <c r="AL18" s="3"/>
+      <c r="AM18" s="3"/>
+      <c r="AN18" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AO18" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AP18" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="AQ18" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="AR18" s="3"/>
+      <c r="AS18" s="3"/>
+      <c r="AT18" s="3"/>
+      <c r="AU18" s="3"/>
+      <c r="AV18" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW18" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="AX18" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="19" spans="1:50">
+      <c r="A19" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="3"/>
+      <c r="M19" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N19" s="3">
+        <v>13</v>
+      </c>
+      <c r="O19" s="3"/>
+      <c r="P19" s="3"/>
+      <c r="Q19" s="3"/>
+      <c r="R19" s="3">
+        <v>180</v>
+      </c>
+      <c r="S19" s="3"/>
+      <c r="T19" s="3"/>
+      <c r="U19" s="3"/>
+      <c r="V19" s="3">
+        <v>360</v>
+      </c>
+      <c r="W19" s="3"/>
+      <c r="X19" s="3"/>
+      <c r="Y19" s="3">
+        <v>20</v>
+      </c>
+      <c r="Z19" s="3"/>
+      <c r="AA19" s="3"/>
+      <c r="AB19" s="3"/>
+      <c r="AC19" s="3"/>
+      <c r="AD19" s="3"/>
+      <c r="AE19" s="3"/>
+      <c r="AF19" s="3"/>
+      <c r="AG19" s="3"/>
+      <c r="AH19" s="3"/>
+      <c r="AI19" s="3"/>
+      <c r="AJ19" s="3"/>
+      <c r="AK19" s="3"/>
+      <c r="AL19" s="3"/>
+      <c r="AM19" s="3"/>
+      <c r="AN19" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AO19" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AP19" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="AQ19" s="3"/>
+      <c r="AR19" s="3"/>
+      <c r="AS19" s="3"/>
+      <c r="AT19" s="3"/>
+      <c r="AU19" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="AV19" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW19" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="AX19" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="20" spans="1:50">
+      <c r="A20" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
+      <c r="M20" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N20" s="3">
+        <v>13</v>
+      </c>
+      <c r="O20" s="3"/>
+      <c r="P20" s="3"/>
+      <c r="Q20" s="3"/>
+      <c r="R20" s="3">
+        <v>180</v>
+      </c>
+      <c r="S20" s="3"/>
+      <c r="T20" s="3"/>
+      <c r="U20" s="3"/>
+      <c r="V20" s="3">
+        <v>360</v>
+      </c>
+      <c r="W20" s="3"/>
+      <c r="X20" s="3"/>
+      <c r="Y20" s="3">
+        <v>20</v>
+      </c>
+      <c r="Z20" s="3"/>
+      <c r="AA20" s="3"/>
+      <c r="AB20" s="3"/>
+      <c r="AC20" s="3"/>
+      <c r="AD20" s="3"/>
+      <c r="AE20" s="3"/>
+      <c r="AF20" s="3"/>
+      <c r="AG20" s="3"/>
+      <c r="AH20" s="3"/>
+      <c r="AI20" s="3"/>
+      <c r="AJ20" s="3"/>
+      <c r="AK20" s="3"/>
+      <c r="AL20" s="3"/>
+      <c r="AM20" s="3"/>
+      <c r="AN20" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AO20" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AP20" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="AQ20" s="3"/>
+      <c r="AR20" s="3"/>
+      <c r="AS20" s="3"/>
+      <c r="AT20" s="3"/>
+      <c r="AU20" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="AV20" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW20" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="AX20" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC0DE945-E06A-4516-B67F-01CC5F88B8E8}">
+  <dimension ref="A1:C42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
+  <cols>
+    <col min="1" max="1" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="82.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1">
+      <c r="A30" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1">
+      <c r="A32" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1">
+      <c r="A36" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1">
+      <c r="A40" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1">
+      <c r="A41" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>